<commit_message>
added tier 6 runics
</commit_message>
<xml_diff>
--- a/The Runics 符灵 Alpha_Data/StreamingAssets/runics.xlsx
+++ b/The Runics 符灵 Alpha_Data/StreamingAssets/runics.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="120">
   <si>
     <t>RunicID</t>
   </si>
@@ -374,6 +374,21 @@
   </si>
   <si>
     <t>Awaken</t>
+  </si>
+  <si>
+    <t>Archill</t>
+  </si>
+  <si>
+    <t>IceStorm</t>
+  </si>
+  <si>
+    <t>TheDemon</t>
+  </si>
+  <si>
+    <t>Demon</t>
+  </si>
+  <si>
+    <t>FirePossession</t>
   </si>
 </sst>
 </file>
@@ -1304,7 +1319,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="C7:O179"/>
+  <dimension ref="C7:O187"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="7" max="7" width="13.2727272727273" customWidth="1"/>
@@ -4446,6 +4461,150 @@
         <v>0.4</v>
       </c>
       <c r="H179">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="181" spans="3:13">
+      <c r="C181" t="s">
+        <v>0</v>
+      </c>
+      <c r="D181" t="s">
+        <v>115</v>
+      </c>
+      <c r="E181" t="s">
+        <v>2</v>
+      </c>
+      <c r="F181">
+        <v>6</v>
+      </c>
+      <c r="G181" t="s">
+        <v>3</v>
+      </c>
+      <c r="H181" t="s">
+        <v>16</v>
+      </c>
+      <c r="I181" t="s">
+        <v>5</v>
+      </c>
+      <c r="J181" t="s">
+        <v>30</v>
+      </c>
+      <c r="L181" t="s">
+        <v>7</v>
+      </c>
+      <c r="M181" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="182" spans="3:8">
+      <c r="C182" t="s">
+        <v>9</v>
+      </c>
+      <c r="D182" t="s">
+        <v>10</v>
+      </c>
+      <c r="E182" t="s">
+        <v>11</v>
+      </c>
+      <c r="F182" t="s">
+        <v>12</v>
+      </c>
+      <c r="G182" t="s">
+        <v>13</v>
+      </c>
+      <c r="H182" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="183" spans="3:8">
+      <c r="C183">
+        <v>32</v>
+      </c>
+      <c r="D183">
+        <v>6</v>
+      </c>
+      <c r="E183">
+        <v>298</v>
+      </c>
+      <c r="F183">
+        <v>4</v>
+      </c>
+      <c r="G183">
+        <v>0.4</v>
+      </c>
+      <c r="H183">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="185" spans="3:13">
+      <c r="C185" t="s">
+        <v>0</v>
+      </c>
+      <c r="D185" t="s">
+        <v>117</v>
+      </c>
+      <c r="E185" t="s">
+        <v>2</v>
+      </c>
+      <c r="F185">
+        <v>6</v>
+      </c>
+      <c r="G185" t="s">
+        <v>3</v>
+      </c>
+      <c r="H185" t="s">
+        <v>4</v>
+      </c>
+      <c r="I185" t="s">
+        <v>5</v>
+      </c>
+      <c r="J185" t="s">
+        <v>118</v>
+      </c>
+      <c r="L185" t="s">
+        <v>7</v>
+      </c>
+      <c r="M185" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="186" spans="3:8">
+      <c r="C186" t="s">
+        <v>9</v>
+      </c>
+      <c r="D186" t="s">
+        <v>10</v>
+      </c>
+      <c r="E186" t="s">
+        <v>11</v>
+      </c>
+      <c r="F186" t="s">
+        <v>12</v>
+      </c>
+      <c r="G186" t="s">
+        <v>13</v>
+      </c>
+      <c r="H186" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="187" spans="3:8">
+      <c r="C187">
+        <v>34</v>
+      </c>
+      <c r="D187">
+        <v>8</v>
+      </c>
+      <c r="E187">
+        <v>305</v>
+      </c>
+      <c r="F187">
+        <v>3</v>
+      </c>
+      <c r="G187">
+        <v>0.5</v>
+      </c>
+      <c r="H187">
         <v>-1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Card pack system and tier 6 runics
</commit_message>
<xml_diff>
--- a/The Runics 符灵 Alpha_Data/StreamingAssets/runics.xlsx
+++ b/The Runics 符灵 Alpha_Data/StreamingAssets/runics.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="130">
   <si>
     <t>RunicID</t>
   </si>
@@ -389,6 +389,36 @@
   </si>
   <si>
     <t>FirePossession</t>
+  </si>
+  <si>
+    <t>LightDragon</t>
+  </si>
+  <si>
+    <t>Heaven</t>
+  </si>
+  <si>
+    <t>AncientWind</t>
+  </si>
+  <si>
+    <t>WindRider</t>
+  </si>
+  <si>
+    <t>SunChaser</t>
+  </si>
+  <si>
+    <t>SunChasing</t>
+  </si>
+  <si>
+    <t>WorldTree</t>
+  </si>
+  <si>
+    <t>WorldFavour</t>
+  </si>
+  <si>
+    <t>EnderHunter</t>
+  </si>
+  <si>
+    <t>EnderShot</t>
   </si>
 </sst>
 </file>
@@ -1319,7 +1349,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="C7:O187"/>
+  <dimension ref="C7:O207"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="7" max="7" width="13.2727272727273" customWidth="1"/>
@@ -4337,7 +4367,7 @@
         <v>3</v>
       </c>
       <c r="J173" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="K173" t="s">
         <v>5</v>
@@ -4487,7 +4517,7 @@
         <v>5</v>
       </c>
       <c r="J181" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="L181" t="s">
         <v>7</v>
@@ -4606,6 +4636,366 @@
       </c>
       <c r="H187">
         <v>-1</v>
+      </c>
+    </row>
+    <row r="189" spans="3:13">
+      <c r="C189" t="s">
+        <v>0</v>
+      </c>
+      <c r="D189" t="s">
+        <v>120</v>
+      </c>
+      <c r="E189" t="s">
+        <v>2</v>
+      </c>
+      <c r="F189">
+        <v>4</v>
+      </c>
+      <c r="G189" t="s">
+        <v>3</v>
+      </c>
+      <c r="H189" t="s">
+        <v>58</v>
+      </c>
+      <c r="I189" t="s">
+        <v>5</v>
+      </c>
+      <c r="J189" t="s">
+        <v>35</v>
+      </c>
+      <c r="L189" t="s">
+        <v>7</v>
+      </c>
+      <c r="M189" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="190" spans="3:8">
+      <c r="C190" t="s">
+        <v>9</v>
+      </c>
+      <c r="D190" t="s">
+        <v>10</v>
+      </c>
+      <c r="E190" t="s">
+        <v>11</v>
+      </c>
+      <c r="F190" t="s">
+        <v>12</v>
+      </c>
+      <c r="G190" t="s">
+        <v>13</v>
+      </c>
+      <c r="H190" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="191" spans="3:8">
+      <c r="C191">
+        <v>21</v>
+      </c>
+      <c r="D191">
+        <v>5</v>
+      </c>
+      <c r="E191">
+        <v>188</v>
+      </c>
+      <c r="F191">
+        <v>3</v>
+      </c>
+      <c r="G191">
+        <v>0.5</v>
+      </c>
+      <c r="H191">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="193" spans="3:13">
+      <c r="C193" t="s">
+        <v>0</v>
+      </c>
+      <c r="D193" t="s">
+        <v>122</v>
+      </c>
+      <c r="E193" t="s">
+        <v>2</v>
+      </c>
+      <c r="F193">
+        <v>6</v>
+      </c>
+      <c r="G193" t="s">
+        <v>3</v>
+      </c>
+      <c r="H193" t="s">
+        <v>20</v>
+      </c>
+      <c r="I193" t="s">
+        <v>5</v>
+      </c>
+      <c r="J193" t="s">
+        <v>30</v>
+      </c>
+      <c r="L193" t="s">
+        <v>7</v>
+      </c>
+      <c r="M193" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="194" spans="3:8">
+      <c r="C194" t="s">
+        <v>9</v>
+      </c>
+      <c r="D194" t="s">
+        <v>10</v>
+      </c>
+      <c r="E194" t="s">
+        <v>11</v>
+      </c>
+      <c r="F194" t="s">
+        <v>12</v>
+      </c>
+      <c r="G194" t="s">
+        <v>13</v>
+      </c>
+      <c r="H194" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="195" spans="3:8">
+      <c r="C195">
+        <v>26</v>
+      </c>
+      <c r="D195">
+        <v>6</v>
+      </c>
+      <c r="E195">
+        <v>266</v>
+      </c>
+      <c r="F195">
+        <v>4</v>
+      </c>
+      <c r="G195">
+        <v>0.4</v>
+      </c>
+      <c r="H195">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="197" spans="3:13">
+      <c r="C197" t="s">
+        <v>0</v>
+      </c>
+      <c r="D197" t="s">
+        <v>124</v>
+      </c>
+      <c r="E197" t="s">
+        <v>2</v>
+      </c>
+      <c r="F197">
+        <v>6</v>
+      </c>
+      <c r="G197" t="s">
+        <v>3</v>
+      </c>
+      <c r="H197" t="s">
+        <v>34</v>
+      </c>
+      <c r="I197" t="s">
+        <v>5</v>
+      </c>
+      <c r="J197" t="s">
+        <v>6</v>
+      </c>
+      <c r="L197" t="s">
+        <v>7</v>
+      </c>
+      <c r="M197" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="198" spans="3:8">
+      <c r="C198" t="s">
+        <v>9</v>
+      </c>
+      <c r="D198" t="s">
+        <v>10</v>
+      </c>
+      <c r="E198" t="s">
+        <v>11</v>
+      </c>
+      <c r="F198" t="s">
+        <v>12</v>
+      </c>
+      <c r="G198" t="s">
+        <v>13</v>
+      </c>
+      <c r="H198" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="199" spans="3:8">
+      <c r="C199">
+        <v>34</v>
+      </c>
+      <c r="D199">
+        <v>7</v>
+      </c>
+      <c r="E199">
+        <v>285</v>
+      </c>
+      <c r="F199">
+        <v>4</v>
+      </c>
+      <c r="G199">
+        <v>0.4</v>
+      </c>
+      <c r="H199">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="201" spans="3:13">
+      <c r="C201" t="s">
+        <v>0</v>
+      </c>
+      <c r="D201" t="s">
+        <v>126</v>
+      </c>
+      <c r="E201" t="s">
+        <v>2</v>
+      </c>
+      <c r="F201">
+        <v>6</v>
+      </c>
+      <c r="G201" t="s">
+        <v>3</v>
+      </c>
+      <c r="H201" t="s">
+        <v>50</v>
+      </c>
+      <c r="I201" t="s">
+        <v>5</v>
+      </c>
+      <c r="J201" t="s">
+        <v>35</v>
+      </c>
+      <c r="L201" t="s">
+        <v>7</v>
+      </c>
+      <c r="M201" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="202" spans="3:8">
+      <c r="C202" t="s">
+        <v>9</v>
+      </c>
+      <c r="D202" t="s">
+        <v>10</v>
+      </c>
+      <c r="E202" t="s">
+        <v>11</v>
+      </c>
+      <c r="F202" t="s">
+        <v>12</v>
+      </c>
+      <c r="G202" t="s">
+        <v>13</v>
+      </c>
+      <c r="H202" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="203" spans="3:8">
+      <c r="C203">
+        <v>28</v>
+      </c>
+      <c r="D203">
+        <v>8</v>
+      </c>
+      <c r="E203">
+        <v>325</v>
+      </c>
+      <c r="F203">
+        <v>3</v>
+      </c>
+      <c r="G203">
+        <v>0.5</v>
+      </c>
+      <c r="H203">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="205" spans="3:13">
+      <c r="C205" t="s">
+        <v>0</v>
+      </c>
+      <c r="D205" t="s">
+        <v>128</v>
+      </c>
+      <c r="E205" t="s">
+        <v>2</v>
+      </c>
+      <c r="F205">
+        <v>6</v>
+      </c>
+      <c r="G205" t="s">
+        <v>3</v>
+      </c>
+      <c r="H205" t="s">
+        <v>16</v>
+      </c>
+      <c r="I205" t="s">
+        <v>5</v>
+      </c>
+      <c r="J205" t="s">
+        <v>63</v>
+      </c>
+      <c r="L205" t="s">
+        <v>7</v>
+      </c>
+      <c r="M205" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="206" spans="3:8">
+      <c r="C206" t="s">
+        <v>9</v>
+      </c>
+      <c r="D206" t="s">
+        <v>10</v>
+      </c>
+      <c r="E206" t="s">
+        <v>11</v>
+      </c>
+      <c r="F206" t="s">
+        <v>12</v>
+      </c>
+      <c r="G206" t="s">
+        <v>13</v>
+      </c>
+      <c r="H206" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="207" spans="3:8">
+      <c r="C207">
+        <v>32</v>
+      </c>
+      <c r="D207">
+        <v>6</v>
+      </c>
+      <c r="E207">
+        <v>285</v>
+      </c>
+      <c r="F207">
+        <v>5</v>
+      </c>
+      <c r="G207">
+        <v>0.4</v>
+      </c>
+      <c r="H207">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>